<commit_message>
Correct rate sensitivity scope in lender model
</commit_message>
<xml_diff>
--- a/model/Morrisons_Leveraged_Finance_Model.xlsx
+++ b/model/Morrisons_Leveraged_Finance_Model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R09b23359ee374066"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Ra51f6379c0c84ee4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical" sheetId="3" r:id="Rcbef3ec1000c4bec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base Case" sheetId="4" r:id="R8e53c628588c4c2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Downside" sheetId="5" r:id="Rdec4851c4da947a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt Capacity" sheetId="6" r:id="R92ad416743ec4fc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Checks" sheetId="7" r:id="Red6b11b7ab984d53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R4f6093fe3f594d6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R134e26beb31e401b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical" sheetId="3" r:id="R2a25c40707404aa1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base Case" sheetId="4" r:id="R4e61f8d417d44869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Downside" sheetId="5" r:id="Rc9766d1c088a487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt Capacity" sheetId="6" r:id="R29326eecb20a476d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Checks" sheetId="7" r:id="R3f44474651b94715"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1536,7 +1536,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R21c7c4baa4cb4e51"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R02b64bf2e72b4a06"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1566,7 +1566,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R941020c5e2d54ee5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1e32ef5961394586"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3874,7 +3874,7 @@
     <x:mergeCell ref="A39:Q40"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a3657b3fdbc4bd5"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bb13cd8d6534401"/>
 </x:worksheet>
 </file>
 
@@ -8289,7 +8289,7 @@
       <x:c r="C40" s="102"/>
       <x:c r="D40" s="102"/>
       <x:c r="E40" s="140" t="str">
-        <x:v>Static FY26 coverage sensitivity: shocks floating term loans only; fixed 2031 notes excluded. No integrated leverage/liquidity reforecast. Commitment fees excluded.</x:v>
+        <x:v>Static FY26 coverage sensitivity: shocks floating existing term loans and proposed term-out; fixed 2031 notes excluded. No integrated leverage/liquidity reforecast. Commitment fees excluded.</x:v>
       </x:c>
       <x:c r="F40" s="140"/>
       <x:c r="G40" s="140"/>
@@ -8446,7 +8446,7 @@
         <x:v>01-Aug-2025</x:v>
       </x:c>
       <x:c r="D6" s="140" t="str">
-        <x:v>FY ended 27-Oct-2024: cash flow p28; interest p57; RCF fees p58; liquidity p63; EBITDA p86</x:v>
+        <x:v>FY ended 27-Oct-2024: cash flow p29; interest p57; RCF fees p58; liquidity p63; EBITDA p86</x:v>
       </x:c>
       <x:c r="E6" s="143" t="str">
         <x:v>https://find-and-update.company-information.service.gov.uk/company/13537474/filing-history/MzQ3NTgxNzc3N2FkaXF6a2N4/document?format=pdf&amp;download=0</x:v>

</xml_diff>